<commit_message>
Cleaned up probability calculations
</commit_message>
<xml_diff>
--- a/statPre/Predictions.xlsx
+++ b/statPre/Predictions.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
   <si>
     <t>Team Against</t>
   </si>
@@ -45,6 +45,18 @@
   </si>
   <si>
     <t>First Name</t>
+  </si>
+  <si>
+    <t>Cleveland Guardians</t>
+  </si>
+  <si>
+    <t>Hernandez</t>
+  </si>
+  <si>
+    <t>Cesar</t>
+  </si>
+  <si>
+    <t>Minnesota Twins</t>
   </si>
 </sst>
 </file>
@@ -89,7 +101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -127,6 +139,76 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="C2" t="n" s="0">
+        <v>76.98</v>
+      </c>
+      <c r="D2" t="n" s="0">
+        <v>0.2619225037257824</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>0.24675324675324675</v>
+      </c>
+      <c r="F2" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="G2" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="H2" t="n" s="0">
+        <v>149.0</v>
+      </c>
+      <c r="I2" t="n" s="0">
+        <v>68.0</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="C3" t="n" s="0">
+        <v>85.03</v>
+      </c>
+      <c r="D3" t="n" s="0">
+        <v>0.7988636363636362</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>0.24675324675324675</v>
+      </c>
+      <c r="F3" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="G3" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="H3" t="n" s="0">
+        <v>149.0</v>
+      </c>
+      <c r="I3" t="n" s="0">
+        <v>68.0</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Deleted unused imports after refactor
</commit_message>
<xml_diff>
--- a/statPre/Predictions.xlsx
+++ b/statPre/Predictions.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="16">
   <si>
     <t>Team Against</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>Minnesota Twins</t>
+  </si>
+  <si>
+    <t>Detroit Tigers</t>
   </si>
 </sst>
 </file>
@@ -101,7 +104,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -209,6 +212,41 @@
         <v>13</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B4" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="C4" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D4" t="n" s="0">
+        <v>0.2619225037257824</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>0.24675324675324675</v>
+      </c>
+      <c r="F4" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="G4" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="H4" t="n" s="0">
+        <v>149.0</v>
+      </c>
+      <c r="I4" t="n" s="0">
+        <v>68.0</v>
+      </c>
+      <c r="J4" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="K4" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>